<commit_message>
pushing after 4 days due to disorganized lifestyle these days
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="375" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE09EABE-76A7-4171-904F-1E909C6481DD}"/>
+  <xr:revisionPtr revIDLastSave="442" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C649ECD3-B54A-495A-92F5-D1F662572D09}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="99">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -314,6 +314,24 @@
   </si>
   <si>
     <t>started studying late due to headache</t>
+  </si>
+  <si>
+    <t>today I ride at 60/70 kmph , didn’t push 80 today</t>
+  </si>
+  <si>
+    <t>due to bike problem less time was dedicated to study</t>
+  </si>
+  <si>
+    <t>today python ca was conducted</t>
+  </si>
+  <si>
+    <t>not able to study due to disorganised sleep cycle</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>not able to study due to disorganised sleep cycle &amp; other chores</t>
   </si>
 </sst>
 </file>
@@ -2430,132 +2448,256 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+    <row r="35" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B35" s="14">
+        <v>600</v>
+      </c>
+      <c r="C35" s="14">
+        <v>100</v>
+      </c>
+      <c r="D35" s="14">
+        <v>0</v>
+      </c>
+      <c r="E35" s="14">
+        <v>0</v>
+      </c>
+      <c r="F35" s="14">
+        <v>0</v>
+      </c>
+      <c r="G35" s="14">
+        <v>0</v>
+      </c>
+      <c r="H35" s="14">
+        <v>630</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1330</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+        <v>110</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B36" s="14">
+        <v>240</v>
+      </c>
+      <c r="C36" s="14">
+        <v>80</v>
+      </c>
+      <c r="D36" s="14">
+        <v>32</v>
+      </c>
+      <c r="E36" s="14">
+        <v>103</v>
+      </c>
+      <c r="F36" s="14">
+        <v>100</v>
+      </c>
+      <c r="G36" s="14">
+        <v>2</v>
+      </c>
+      <c r="H36" s="14">
+        <v>520</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1075</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
+        <v>365</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B37" s="14">
+        <v>270</v>
+      </c>
+      <c r="C37" s="14">
+        <v>80</v>
+      </c>
+      <c r="D37" s="14">
+        <v>45</v>
+      </c>
+      <c r="E37" s="14">
+        <v>90</v>
+      </c>
+      <c r="F37" s="14">
+        <v>250</v>
+      </c>
+      <c r="G37" s="14">
+        <v>5</v>
+      </c>
+      <c r="H37" s="14">
+        <v>320</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>1055</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+        <v>385</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B38" s="14">
+        <v>287</v>
+      </c>
+      <c r="C38" s="14">
+        <v>140</v>
+      </c>
+      <c r="D38" s="14">
+        <v>0</v>
+      </c>
+      <c r="E38" s="14">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14">
+        <v>150</v>
+      </c>
+      <c r="G38" s="14">
+        <v>3</v>
+      </c>
+      <c r="H38" s="14">
+        <v>523</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+        <v>340</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B39" s="14">
+        <v>285</v>
+      </c>
+      <c r="C39" s="14">
+        <v>160</v>
+      </c>
+      <c r="D39" s="14">
+        <v>47</v>
+      </c>
+      <c r="E39" s="14">
+        <v>0</v>
+      </c>
+      <c r="F39" s="14">
+        <v>350</v>
+      </c>
+      <c r="G39" s="14">
+        <v>7</v>
+      </c>
+      <c r="H39" s="14">
+        <v>429</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1271</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
+        <v>169</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
+      <c r="A40" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B40" s="14">
+        <v>287</v>
+      </c>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
       <c r="F40" s="14"/>
       <c r="G40" s="14"/>
       <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>287</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1153</v>
       </c>
       <c r="K40" s="16"/>
       <c r="L40" s="16"/>

</xml_diff>

<commit_message>
pushing after 4,5 days due to being busy
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="522" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44151214-5D18-4276-86C1-43108F6792C1}"/>
+  <xr:revisionPtr revIDLastSave="591" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88B61149-4EB6-44D5-8870-3106D15AA091}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="110">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -350,6 +350,21 @@
   </si>
   <si>
     <t>due to prepration of english ca, I have to skip dinner</t>
+  </si>
+  <si>
+    <t>english ca happens today</t>
+  </si>
+  <si>
+    <t>dbms ca2 happens today, my performance was good</t>
+  </si>
+  <si>
+    <t>I submit python minor project today</t>
+  </si>
+  <si>
+    <t>today I travelled back to room from home but got news that 10 days classes are cancelled due to protest</t>
+  </si>
+  <si>
+    <t>came back home due to classes got cancelled</t>
   </si>
 </sst>
 </file>
@@ -2973,114 +2988,234 @@
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+      <c r="A46" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B46" s="14">
+        <v>331</v>
+      </c>
+      <c r="C46" s="14">
+        <v>80</v>
+      </c>
+      <c r="D46" s="14">
+        <v>135</v>
+      </c>
+      <c r="E46" s="14">
+        <v>224</v>
+      </c>
+      <c r="F46" s="14">
+        <v>350</v>
+      </c>
+      <c r="G46" s="14">
+        <v>7</v>
+      </c>
+      <c r="H46" s="14">
+        <v>234</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>1354</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+        <v>86</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B47" s="14">
+        <v>346</v>
+      </c>
+      <c r="C47" s="14">
+        <v>163</v>
+      </c>
+      <c r="D47" s="14">
+        <v>0</v>
+      </c>
+      <c r="E47" s="14">
+        <v>0</v>
+      </c>
+      <c r="F47" s="14">
+        <v>150</v>
+      </c>
+      <c r="G47" s="14">
+        <v>3</v>
+      </c>
+      <c r="H47" s="14">
+        <v>523</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>1182</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+        <v>258</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N47" s="17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B48" s="14">
+        <v>587</v>
+      </c>
+      <c r="C48" s="14">
+        <v>0</v>
+      </c>
+      <c r="D48" s="14">
+        <v>181</v>
+      </c>
+      <c r="E48" s="14">
+        <v>245</v>
+      </c>
+      <c r="F48" s="14">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14">
+        <v>427</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+        <v>0</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B49" s="14">
+        <v>366</v>
+      </c>
+      <c r="C49" s="14">
+        <v>80</v>
+      </c>
+      <c r="D49" s="14">
+        <v>0</v>
+      </c>
+      <c r="E49" s="14">
+        <v>0</v>
+      </c>
+      <c r="F49" s="14">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14">
+        <v>824</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>1270</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+        <v>170</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B50" s="14">
+        <v>337</v>
+      </c>
+      <c r="C50" s="14">
+        <v>80</v>
+      </c>
+      <c r="D50" s="14">
+        <v>0</v>
+      </c>
+      <c r="E50" s="14">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14">
+        <v>882</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>1299</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
+        <v>141</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>

</xml_diff>

<commit_message>
pushed after 4 days due to being busy
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="823" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C58E405B-7D29-47C6-9EB6-3BE3AD937001}"/>
+  <xr:revisionPtr revIDLastSave="875" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3233D9BD-7FFF-4F38-A1A5-C511A2A29D9D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="130">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -413,6 +413,18 @@
   </si>
   <si>
     <t>maths paper was good and studied for english paper, started dexter</t>
+  </si>
+  <si>
+    <t>went to home after paper</t>
+  </si>
+  <si>
+    <t>watched dexter whole day</t>
+  </si>
+  <si>
+    <t>finished dexter s1 and revise dsa</t>
+  </si>
+  <si>
+    <t>happy dusshera</t>
   </si>
 </sst>
 </file>
@@ -4026,92 +4038,188 @@
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="8"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="10" t="str">
+      <c r="A68" s="8">
+        <v>46312</v>
+      </c>
+      <c r="B68" s="9">
+        <v>347</v>
+      </c>
+      <c r="C68" s="9">
+        <v>102</v>
+      </c>
+      <c r="D68" s="9">
+        <v>156</v>
+      </c>
+      <c r="E68" s="9">
+        <v>0</v>
+      </c>
+      <c r="F68" s="9">
+        <v>0</v>
+      </c>
+      <c r="G68" s="9">
+        <v>0</v>
+      </c>
+      <c r="H68" s="9">
+        <v>835</v>
+      </c>
+      <c r="I68" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="10" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J68" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="11"/>
-      <c r="L68" s="11"/>
-      <c r="M68" s="11"/>
-      <c r="N68" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="K68" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L68" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M68" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N68" s="12" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="8"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="10" t="str">
+      <c r="A69" s="8">
+        <v>46313</v>
+      </c>
+      <c r="B69" s="9">
+        <v>612</v>
+      </c>
+      <c r="C69" s="9">
+        <v>0</v>
+      </c>
+      <c r="D69" s="9">
+        <v>0</v>
+      </c>
+      <c r="E69" s="9">
+        <v>0</v>
+      </c>
+      <c r="F69" s="9">
+        <v>0</v>
+      </c>
+      <c r="G69" s="9">
+        <v>0</v>
+      </c>
+      <c r="H69" s="9">
+        <v>789</v>
+      </c>
+      <c r="I69" s="10">
         <f t="shared" ref="I69:I132" si="2">IF(SUM(B69:F69,H69)=0,"",SUM(B69:F69,H69))</f>
-        <v/>
-      </c>
-      <c r="J69" s="10" t="str">
+        <v>1401</v>
+      </c>
+      <c r="J69" s="10">
         <f t="shared" ref="J69:J132" si="3">IF(I69="","",1440-I69)</f>
-        <v/>
-      </c>
-      <c r="K69" s="11"/>
-      <c r="L69" s="11"/>
-      <c r="M69" s="11"/>
-      <c r="N69" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="K69" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L69" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="M69" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N69" s="12" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="8"/>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="9"/>
-      <c r="F70" s="9"/>
-      <c r="G70" s="9"/>
-      <c r="H70" s="9"/>
-      <c r="I70" s="10" t="str">
+      <c r="A70" s="8">
+        <v>46314</v>
+      </c>
+      <c r="B70" s="9">
+        <v>615</v>
+      </c>
+      <c r="C70" s="9">
+        <v>0</v>
+      </c>
+      <c r="D70" s="9">
+        <v>53</v>
+      </c>
+      <c r="E70" s="9">
+        <v>0</v>
+      </c>
+      <c r="F70" s="9">
+        <v>0</v>
+      </c>
+      <c r="G70" s="9">
+        <v>0</v>
+      </c>
+      <c r="H70" s="9">
+        <v>655</v>
+      </c>
+      <c r="I70" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J70" s="10" t="str">
+        <v>1323</v>
+      </c>
+      <c r="J70" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K70" s="11"/>
-      <c r="L70" s="11"/>
-      <c r="M70" s="11"/>
-      <c r="N70" s="12"/>
+        <v>117</v>
+      </c>
+      <c r="K70" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L70" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="M70" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N70" s="12" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="8"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
-      <c r="F71" s="9"/>
-      <c r="G71" s="9"/>
-      <c r="H71" s="9"/>
-      <c r="I71" s="10" t="str">
+      <c r="A71" s="8">
+        <v>46315</v>
+      </c>
+      <c r="B71" s="9">
+        <v>560</v>
+      </c>
+      <c r="C71" s="9">
+        <v>102</v>
+      </c>
+      <c r="D71" s="9">
+        <v>0</v>
+      </c>
+      <c r="E71" s="9">
+        <v>0</v>
+      </c>
+      <c r="F71" s="9">
+        <v>0</v>
+      </c>
+      <c r="G71" s="9">
+        <v>0</v>
+      </c>
+      <c r="H71" s="9">
+        <v>773</v>
+      </c>
+      <c r="I71" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J71" s="10" t="str">
+        <v>1435</v>
+      </c>
+      <c r="J71" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K71" s="11"/>
-      <c r="L71" s="11"/>
-      <c r="M71" s="11"/>
-      <c r="N71" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="K71" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L71" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="M71" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N71" s="12" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="8"/>

</xml_diff>

<commit_message>
pushed for 2 days
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="875" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3233D9BD-7FFF-4F38-A1A5-C511A2A29D9D}"/>
+  <xr:revisionPtr revIDLastSave="913" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BCC93B-46EE-4DEE-B00B-E82892549FA9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="133">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -425,6 +425,15 @@
   </si>
   <si>
     <t>happy dusshera</t>
+  </si>
+  <si>
+    <t>restarted dsa</t>
+  </si>
+  <si>
+    <t>solved some dsa array questions</t>
+  </si>
+  <si>
+    <t>watched a movie, did rest,re-arrange room</t>
   </si>
 </sst>
 </file>
@@ -4222,70 +4231,142 @@
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="8"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
-      <c r="H72" s="9"/>
-      <c r="I72" s="10" t="str">
+      <c r="A72" s="8">
+        <v>46316</v>
+      </c>
+      <c r="B72" s="9">
+        <v>312</v>
+      </c>
+      <c r="C72" s="9">
+        <v>62</v>
+      </c>
+      <c r="D72" s="9">
+        <v>142</v>
+      </c>
+      <c r="E72" s="9">
+        <v>60</v>
+      </c>
+      <c r="F72" s="9">
+        <v>150</v>
+      </c>
+      <c r="G72" s="9">
+        <v>3</v>
+      </c>
+      <c r="H72" s="9">
+        <v>640</v>
+      </c>
+      <c r="I72" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J72" s="10" t="str">
+        <v>1366</v>
+      </c>
+      <c r="J72" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K72" s="11"/>
-      <c r="L72" s="11"/>
-      <c r="M72" s="11"/>
-      <c r="N72" s="12"/>
+        <v>74</v>
+      </c>
+      <c r="K72" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L72" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M72" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N72" s="12" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="8"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="9"/>
-      <c r="H73" s="9"/>
-      <c r="I73" s="10" t="str">
+      <c r="A73" s="8">
+        <v>46317</v>
+      </c>
+      <c r="B73" s="9">
+        <v>291</v>
+      </c>
+      <c r="C73" s="9">
+        <v>132</v>
+      </c>
+      <c r="D73" s="9">
+        <v>122</v>
+      </c>
+      <c r="E73" s="9">
+        <v>36</v>
+      </c>
+      <c r="F73" s="9">
+        <v>300</v>
+      </c>
+      <c r="G73" s="9">
+        <v>6</v>
+      </c>
+      <c r="H73" s="9">
+        <v>550</v>
+      </c>
+      <c r="I73" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J73" s="10" t="str">
+        <v>1431</v>
+      </c>
+      <c r="J73" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K73" s="11"/>
-      <c r="L73" s="11"/>
-      <c r="M73" s="11"/>
-      <c r="N73" s="12"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A74" s="8"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="9"/>
-      <c r="F74" s="9"/>
-      <c r="G74" s="9"/>
-      <c r="H74" s="9"/>
-      <c r="I74" s="10" t="str">
+        <v>9</v>
+      </c>
+      <c r="K73" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L73" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M73" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N73" s="12" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="8">
+        <v>46318</v>
+      </c>
+      <c r="B74" s="9">
+        <v>381</v>
+      </c>
+      <c r="C74" s="9">
+        <v>45</v>
+      </c>
+      <c r="D74" s="9">
+        <v>0</v>
+      </c>
+      <c r="E74" s="9">
+        <v>0</v>
+      </c>
+      <c r="F74" s="9">
+        <v>250</v>
+      </c>
+      <c r="G74" s="9">
+        <v>5</v>
+      </c>
+      <c r="H74" s="9">
+        <v>621</v>
+      </c>
+      <c r="I74" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J74" s="10" t="str">
+        <v>1297</v>
+      </c>
+      <c r="J74" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K74" s="11"/>
-      <c r="L74" s="11"/>
-      <c r="M74" s="11"/>
-      <c r="N74" s="12"/>
+        <v>143</v>
+      </c>
+      <c r="K74" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L74" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="M74" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N74" s="12" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="8"/>

</xml_diff>

<commit_message>
pushed for 3 days
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="913" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BCC93B-46EE-4DEE-B00B-E82892549FA9}"/>
+  <xr:revisionPtr revIDLastSave="962" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD841695-21D7-47EB-B001-1545B1E1AD0E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="136">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -434,6 +434,15 @@
   </si>
   <si>
     <t>watched a movie, did rest,re-arrange room</t>
+  </si>
+  <si>
+    <t>bought new laptop for business</t>
+  </si>
+  <si>
+    <t>did new laptop setup</t>
+  </si>
+  <si>
+    <t>completed maths test</t>
   </si>
 </sst>
 </file>
@@ -4369,92 +4378,188 @@
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A75" s="8"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="9"/>
-      <c r="G75" s="9"/>
-      <c r="H75" s="9"/>
-      <c r="I75" s="10" t="str">
+      <c r="A75" s="8">
+        <v>46319</v>
+      </c>
+      <c r="B75" s="9">
+        <v>516</v>
+      </c>
+      <c r="C75" s="9">
+        <v>45</v>
+      </c>
+      <c r="D75" s="9">
+        <v>32</v>
+      </c>
+      <c r="E75" s="9">
+        <v>120</v>
+      </c>
+      <c r="F75" s="9">
+        <v>0</v>
+      </c>
+      <c r="G75" s="9">
+        <v>0</v>
+      </c>
+      <c r="H75" s="9">
+        <v>722</v>
+      </c>
+      <c r="I75" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J75" s="10" t="str">
+        <v>1435</v>
+      </c>
+      <c r="J75" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K75" s="11"/>
-      <c r="L75" s="11"/>
-      <c r="M75" s="11"/>
-      <c r="N75" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="K75" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L75" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M75" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N75" s="12" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A76" s="8"/>
-      <c r="B76" s="9"/>
-      <c r="C76" s="9"/>
-      <c r="D76" s="9"/>
-      <c r="E76" s="9"/>
-      <c r="F76" s="9"/>
-      <c r="G76" s="9"/>
-      <c r="H76" s="9"/>
-      <c r="I76" s="10" t="str">
+      <c r="A76" s="8">
+        <v>46320</v>
+      </c>
+      <c r="B76" s="9">
+        <v>516</v>
+      </c>
+      <c r="C76" s="9">
+        <v>0</v>
+      </c>
+      <c r="D76" s="9">
+        <v>92</v>
+      </c>
+      <c r="E76" s="9">
+        <v>0</v>
+      </c>
+      <c r="F76" s="9">
+        <v>0</v>
+      </c>
+      <c r="G76" s="9">
+        <v>0</v>
+      </c>
+      <c r="H76" s="9">
+        <v>755</v>
+      </c>
+      <c r="I76" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J76" s="10" t="str">
+        <v>1363</v>
+      </c>
+      <c r="J76" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K76" s="11"/>
-      <c r="L76" s="11"/>
-      <c r="M76" s="11"/>
-      <c r="N76" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="K76" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L76" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M76" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N76" s="12" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A77" s="8"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="9"/>
-      <c r="F77" s="9"/>
-      <c r="G77" s="9"/>
-      <c r="H77" s="9"/>
-      <c r="I77" s="10" t="str">
+      <c r="A77" s="8">
+        <v>46321</v>
+      </c>
+      <c r="B77" s="9">
+        <v>372</v>
+      </c>
+      <c r="C77" s="9">
+        <v>83</v>
+      </c>
+      <c r="D77" s="9">
+        <v>240</v>
+      </c>
+      <c r="E77" s="9">
+        <v>0</v>
+      </c>
+      <c r="F77" s="9">
+        <v>0</v>
+      </c>
+      <c r="G77" s="9">
+        <v>0</v>
+      </c>
+      <c r="H77" s="9">
+        <v>653</v>
+      </c>
+      <c r="I77" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J77" s="10" t="str">
+        <v>1348</v>
+      </c>
+      <c r="J77" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K77" s="11"/>
-      <c r="L77" s="11"/>
-      <c r="M77" s="11"/>
-      <c r="N77" s="12"/>
+        <v>92</v>
+      </c>
+      <c r="K77" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L77" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M77" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N77" s="12" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A78" s="8"/>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
-      <c r="D78" s="9"/>
-      <c r="E78" s="9"/>
-      <c r="F78" s="9"/>
-      <c r="G78" s="9"/>
-      <c r="H78" s="9"/>
-      <c r="I78" s="10" t="str">
+      <c r="A78" s="8">
+        <v>46322</v>
+      </c>
+      <c r="B78" s="9">
+        <v>362</v>
+      </c>
+      <c r="C78" s="9">
+        <v>122</v>
+      </c>
+      <c r="D78" s="9">
+        <v>120</v>
+      </c>
+      <c r="E78" s="9">
+        <v>0</v>
+      </c>
+      <c r="F78" s="9">
+        <v>250</v>
+      </c>
+      <c r="G78" s="9">
+        <v>5</v>
+      </c>
+      <c r="H78" s="9">
+        <v>520</v>
+      </c>
+      <c r="I78" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J78" s="10" t="str">
+        <v>1374</v>
+      </c>
+      <c r="J78" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K78" s="11"/>
-      <c r="L78" s="11"/>
-      <c r="M78" s="11"/>
-      <c r="N78" s="12"/>
+        <v>66</v>
+      </c>
+      <c r="K78" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L78" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M78" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N78" s="12" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" s="8"/>

</xml_diff>

<commit_message>
pushed for 2 days , and early push for today
</commit_message>
<xml_diff>
--- a/12603996.xlsx
+++ b/12603996.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lpuin-my.sharepoint.com/personal/shubham_bither2026_lpu_in/Documents/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="962" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD841695-21D7-47EB-B001-1545B1E1AD0E}"/>
+  <xr:revisionPtr revIDLastSave="998" documentId="8_{04F8DF2E-49C5-3B44-B164-C4F738DF63B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEC7639B-FFD0-4C70-BBB5-94C100A5A163}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="138">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -443,6 +443,12 @@
   </si>
   <si>
     <t>completed maths test</t>
+  </si>
+  <si>
+    <t>prepared for ca2 of networking</t>
+  </si>
+  <si>
+    <t>went to home ,did c++ project preparation</t>
   </si>
 </sst>
 </file>
@@ -4562,70 +4568,138 @@
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A79" s="8"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="9"/>
-      <c r="F79" s="9"/>
-      <c r="G79" s="9"/>
-      <c r="H79" s="9"/>
-      <c r="I79" s="10" t="str">
+      <c r="A79" s="8">
+        <v>46323</v>
+      </c>
+      <c r="B79" s="9">
+        <v>332</v>
+      </c>
+      <c r="C79" s="9">
+        <v>152</v>
+      </c>
+      <c r="D79" s="9">
+        <v>180</v>
+      </c>
+      <c r="E79" s="9">
+        <v>0</v>
+      </c>
+      <c r="F79" s="9">
+        <v>150</v>
+      </c>
+      <c r="G79" s="9">
+        <v>3</v>
+      </c>
+      <c r="H79" s="9">
+        <v>561</v>
+      </c>
+      <c r="I79" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J79" s="10" t="str">
+        <v>1375</v>
+      </c>
+      <c r="J79" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K79" s="11"/>
-      <c r="L79" s="11"/>
-      <c r="M79" s="11"/>
-      <c r="N79" s="12"/>
+        <v>65</v>
+      </c>
+      <c r="K79" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L79" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M79" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N79" s="12" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A80" s="8"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="9"/>
-      <c r="D80" s="9"/>
-      <c r="E80" s="9"/>
-      <c r="F80" s="9"/>
-      <c r="G80" s="9"/>
-      <c r="H80" s="9"/>
-      <c r="I80" s="10" t="str">
+      <c r="A80" s="8">
+        <v>46324</v>
+      </c>
+      <c r="B80" s="9">
+        <v>332</v>
+      </c>
+      <c r="C80" s="9">
+        <v>89</v>
+      </c>
+      <c r="D80" s="9">
+        <v>240</v>
+      </c>
+      <c r="E80" s="9">
+        <v>0</v>
+      </c>
+      <c r="F80" s="9">
+        <v>250</v>
+      </c>
+      <c r="G80" s="9">
+        <v>5</v>
+      </c>
+      <c r="H80" s="9">
+        <v>529</v>
+      </c>
+      <c r="I80" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J80" s="10" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J80" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K80" s="11"/>
-      <c r="L80" s="11"/>
-      <c r="M80" s="11"/>
-      <c r="N80" s="12"/>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A81" s="8"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
-      <c r="D81" s="9"/>
+        <v>0</v>
+      </c>
+      <c r="K80" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L80" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="M80" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N80" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A81" s="8">
+        <v>46325</v>
+      </c>
+      <c r="B81" s="9">
+        <v>332</v>
+      </c>
+      <c r="C81" s="9">
+        <v>132</v>
+      </c>
+      <c r="D81" s="9">
+        <v>82</v>
+      </c>
       <c r="E81" s="9"/>
-      <c r="F81" s="9"/>
-      <c r="G81" s="9"/>
+      <c r="F81" s="9">
+        <v>250</v>
+      </c>
+      <c r="G81" s="9">
+        <v>5</v>
+      </c>
       <c r="H81" s="9"/>
-      <c r="I81" s="10" t="str">
+      <c r="I81" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J81" s="10" t="str">
+        <v>796</v>
+      </c>
+      <c r="J81" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K81" s="11"/>
-      <c r="L81" s="11"/>
-      <c r="M81" s="11"/>
-      <c r="N81" s="12"/>
+        <v>644</v>
+      </c>
+      <c r="K81" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L81" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M81" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="N81" s="12" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="8"/>

</xml_diff>